<commit_message>
Add support for <br>-style line breaks in analysis tools
</commit_message>
<xml_diff>
--- a/code-analysis/word-count-deep-dives/Deep-dives-word-counts.xlsx
+++ b/code-analysis/word-count-deep-dives/Deep-dives-word-counts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mark/Documents/Files/Websites/Repositories/bbcelite-scripts/code-analysis/word-count-deep-dives/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E00941E6-9178-9948-860E-1C5748E1770C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4334C6B3-F0CE-8F4D-B2A5-1616DFD92500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15540" yWindow="2540" windowWidth="19940" windowHeight="17440" xr2:uid="{B861FA09-B3AD-9448-956B-DECF27F030C1}"/>
   </bookViews>
@@ -1322,11 +1322,11 @@
       </c>
       <c r="B2" s="4">
         <f>SUMIF(wordcount.txt!B:B,"*elite.bbcelite.com*",wordcount.txt!A:A)</f>
-        <v>229655</v>
+        <v>229851</v>
       </c>
       <c r="C2" s="6">
         <f>B2/$B$8</f>
-        <v>0.41808589461879736</v>
+        <v>0.41754271233548595</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -1335,11 +1335,11 @@
       </c>
       <c r="B3" s="4">
         <f>SUMIF(wordcount.txt!B:B,"*revs.bbcelite.com*",wordcount.txt!A:A)</f>
-        <v>125524</v>
+        <v>126205</v>
       </c>
       <c r="C3" s="6">
         <f>B3/$B$8</f>
-        <v>0.22851587745152477</v>
+        <v>0.2292614694315013</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1348,11 +1348,11 @@
       </c>
       <c r="B4" s="4">
         <f>SUMIF(wordcount.txt!B:B,"*thesentinel.bbcelite.com*",wordcount.txt!A:A)</f>
-        <v>116022</v>
+        <v>116240</v>
       </c>
       <c r="C4" s="6">
         <f>B4/$B$8</f>
-        <v>0.21121752918709413</v>
+        <v>0.21115925047912296</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -1361,11 +1361,11 @@
       </c>
       <c r="B5" s="4">
         <f>SUMIF(wordcount.txt!B:B,"*aviator.bbcelite.com*",wordcount.txt!A:A)</f>
-        <v>41357</v>
+        <v>41401</v>
       </c>
       <c r="C5" s="6">
         <f>B5/$B$8</f>
-        <v>7.5290232495480613E-2</v>
+        <v>7.5208225473900284E-2</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -1374,11 +1374,11 @@
       </c>
       <c r="B6" s="4">
         <f>SUMIF(wordcount.txt!B:B,"*lander.bbcelite.com*",wordcount.txt!A:A)</f>
-        <v>36743</v>
+        <v>36788</v>
       </c>
       <c r="C6" s="6">
         <f>B6/$B$8</f>
-        <v>6.6890466247103139E-2</v>
+        <v>6.6828342279989461E-2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="B8" s="5">
         <f>SUM(B2:B6)</f>
-        <v>549301</v>
+        <v>550485</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -1463,7 +1463,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
-        <v>3370</v>
+        <v>3402</v>
       </c>
       <c r="B7" t="s">
         <v>223</v>
@@ -1471,7 +1471,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
-        <v>3191</v>
+        <v>3201</v>
       </c>
       <c r="B8" t="s">
         <v>238</v>
@@ -1511,7 +1511,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <v>2862</v>
+        <v>2863</v>
       </c>
       <c r="B13" t="s">
         <v>17</v>
@@ -1527,7 +1527,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>2817</v>
+        <v>2826</v>
       </c>
       <c r="B15" t="s">
         <v>15</v>
@@ -1559,7 +1559,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>2638</v>
+        <v>2650</v>
       </c>
       <c r="B19" t="s">
         <v>18</v>
@@ -1575,18 +1575,18 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>2582</v>
+        <v>2607</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>2569</v>
+        <v>2582</v>
       </c>
       <c r="B22" t="s">
-        <v>240</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -1703,7 +1703,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
-        <v>2097</v>
+        <v>2134</v>
       </c>
       <c r="B37" t="s">
         <v>227</v>
@@ -1767,7 +1767,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
-        <v>1887</v>
+        <v>1894</v>
       </c>
       <c r="B45" t="s">
         <v>36</v>
@@ -2151,66 +2151,66 @@
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
-        <v>1076</v>
+        <v>1089</v>
       </c>
       <c r="B93" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
-        <v>1071</v>
+        <v>1076</v>
       </c>
       <c r="B94" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
-        <v>1032</v>
+        <v>1040</v>
       </c>
       <c r="B95" t="s">
-        <v>82</v>
+        <v>113</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="B96" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="B97" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
-        <v>1023</v>
+        <v>1027</v>
       </c>
       <c r="B98" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
-        <v>1018</v>
+        <v>1023</v>
       </c>
       <c r="B99" t="s">
-        <v>233</v>
+        <v>84</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
-        <v>1014</v>
+        <v>1018</v>
       </c>
       <c r="B100" t="s">
-        <v>113</v>
+        <v>233</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
@@ -2391,18 +2391,18 @@
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A123" s="1">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B123" t="s">
-        <v>107</v>
+        <v>235</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A124" s="1">
-        <v>552</v>
+        <v>557</v>
       </c>
       <c r="B124" t="s">
-        <v>235</v>
+        <v>107</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.2">
@@ -2471,7 +2471,7 @@
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A133" s="1">
-        <v>7325</v>
+        <v>7326</v>
       </c>
       <c r="B133" t="s">
         <v>118</v>
@@ -2495,7 +2495,7 @@
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" s="1">
-        <v>4854</v>
+        <v>4858</v>
       </c>
       <c r="B136" t="s">
         <v>121</v>
@@ -2519,7 +2519,7 @@
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" s="1">
-        <v>4659</v>
+        <v>4682</v>
       </c>
       <c r="B139" t="s">
         <v>124</v>
@@ -2543,7 +2543,7 @@
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A142" s="1">
-        <v>3684</v>
+        <v>3688</v>
       </c>
       <c r="B142" t="s">
         <v>127</v>
@@ -2559,7 +2559,7 @@
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A144" s="1">
-        <v>3627</v>
+        <v>3640</v>
       </c>
       <c r="B144" t="s">
         <v>129</v>
@@ -2575,31 +2575,31 @@
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A146" s="1">
-        <v>3178</v>
+        <v>3267</v>
       </c>
       <c r="B146" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A147" s="1">
-        <v>3168</v>
+        <v>3208</v>
       </c>
       <c r="B147" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A148" s="1">
-        <v>3109</v>
+        <v>3178</v>
       </c>
       <c r="B148" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A149" s="1">
-        <v>3057</v>
+        <v>3156</v>
       </c>
       <c r="B149" t="s">
         <v>134</v>
@@ -2607,7 +2607,7 @@
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A150" s="1">
-        <v>2975</v>
+        <v>3074</v>
       </c>
       <c r="B150" t="s">
         <v>135</v>
@@ -2615,34 +2615,34 @@
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A151" s="1">
-        <v>2923</v>
+        <v>3007</v>
       </c>
       <c r="B151" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A152" s="1">
-        <v>2908</v>
+        <v>2923</v>
       </c>
       <c r="B152" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A153" s="1">
-        <v>2852</v>
+        <v>2857</v>
       </c>
       <c r="B153" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A154" s="1">
-        <v>2758</v>
+        <v>2852</v>
       </c>
       <c r="B154" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.2">
@@ -2695,18 +2695,18 @@
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A161" s="1">
-        <v>1878</v>
+        <v>1893</v>
       </c>
       <c r="B161" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A162" s="1">
-        <v>1851</v>
+        <v>1878</v>
       </c>
       <c r="B162" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.2">
@@ -2879,7 +2879,7 @@
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A184" s="1">
-        <v>2536</v>
+        <v>2539</v>
       </c>
       <c r="B184" t="s">
         <v>170</v>
@@ -2911,7 +2911,7 @@
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A188" s="1">
-        <v>1548</v>
+        <v>1587</v>
       </c>
       <c r="B188" t="s">
         <v>173</v>
@@ -3023,7 +3023,7 @@
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A202" s="1">
-        <v>1137</v>
+        <v>1139</v>
       </c>
       <c r="B202" t="s">
         <v>187</v>
@@ -3151,7 +3151,7 @@
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A218" s="1">
-        <v>4682</v>
+        <v>4684</v>
       </c>
       <c r="B218" t="s">
         <v>294</v>
@@ -3175,18 +3175,18 @@
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A221" s="1">
-        <v>3804</v>
+        <v>3864</v>
       </c>
       <c r="B221" t="s">
-        <v>293</v>
+        <v>273</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A222" s="1">
-        <v>3788</v>
+        <v>3808</v>
       </c>
       <c r="B222" t="s">
-        <v>273</v>
+        <v>293</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.2">
@@ -3223,7 +3223,7 @@
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A227" s="1">
-        <v>3046</v>
+        <v>3050</v>
       </c>
       <c r="B227" t="s">
         <v>270</v>
@@ -3247,7 +3247,7 @@
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A230" s="1">
-        <v>2799</v>
+        <v>2814</v>
       </c>
       <c r="B230" t="s">
         <v>266</v>
@@ -3399,26 +3399,26 @@
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A249" s="1">
-        <v>1501</v>
+        <v>1518</v>
       </c>
       <c r="B249" t="s">
-        <v>251</v>
+        <v>267</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A250" s="1">
-        <v>1500</v>
+        <v>1514</v>
       </c>
       <c r="B250" t="s">
-        <v>267</v>
+        <v>252</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A251" s="1">
-        <v>1448</v>
+        <v>1501</v>
       </c>
       <c r="B251" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.2">
@@ -3487,18 +3487,18 @@
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A260" s="1">
-        <v>976</v>
+        <v>992</v>
       </c>
       <c r="B260" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A261" s="1">
-        <v>959</v>
+        <v>976</v>
       </c>
       <c r="B261" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.2">
@@ -3543,7 +3543,7 @@
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A267" s="1">
-        <v>3234</v>
+        <v>3252</v>
       </c>
       <c r="B267" t="s">
         <v>200</v>
@@ -3591,7 +3591,7 @@
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A273" s="1">
-        <v>2606</v>
+        <v>2613</v>
       </c>
       <c r="B273" t="s">
         <v>205</v>
@@ -3631,7 +3631,7 @@
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A278" s="1">
-        <v>1417</v>
+        <v>1424</v>
       </c>
       <c r="B278" t="s">
         <v>210</v>
@@ -3647,7 +3647,7 @@
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A280" s="1">
-        <v>1024</v>
+        <v>1037</v>
       </c>
       <c r="B280" t="s">
         <v>213</v>

</xml_diff>